<commit_message>
Add cooking result management feature
</commit_message>
<xml_diff>
--- a/CurryRecipeManager/docs/01_design/105システムフロー.xlsx
+++ b/CurryRecipeManager/docs/01_design/105システムフロー.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="18551" windowHeight="9840" activeTab="1"/>
+    <workbookView windowWidth="22451" windowHeight="9900" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="レシピ一覧" sheetId="2" r:id="rId1"/>
@@ -141,6 +141,43 @@
     </font>
     <font>
       <sz val="11"/>
+      <color indexed="8"/>
+      <name val="ＭＳ Ｐゴシック"/>
+      <charset val="128"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="ＭＳ Ｐゴシック"/>
+      <charset val="128"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="ＭＳ Ｐゴシック"/>
+      <charset val="128"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="ＭＳ Ｐゴシック"/>
+      <charset val="128"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="ＭＳ Ｐゴシック"/>
+      <charset val="128"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="ＭＳ Ｐゴシック"/>
       <charset val="128"/>
@@ -155,22 +192,8 @@
     </font>
     <font>
       <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="ＭＳ Ｐゴシック"/>
-      <charset val="128"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <sz val="11"/>
-      <color indexed="8"/>
-      <name val="ＭＳ Ｐゴシック"/>
-      <charset val="128"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
+      <color rgb="FF3F3F3F"/>
       <name val="ＭＳ Ｐゴシック"/>
       <charset val="128"/>
       <scheme val="minor"/>
@@ -184,16 +207,25 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="ＭＳ Ｐゴシック"/>
+      <charset val="128"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <b/>
-      <sz val="11"/>
+      <sz val="13"/>
       <color theme="3"/>
       <name val="ＭＳ Ｐゴシック"/>
       <charset val="128"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <u/>
       <sz val="11"/>
-      <color rgb="FFFA7D00"/>
+      <color rgb="FF800080"/>
       <name val="ＭＳ Ｐゴシック"/>
       <charset val="128"/>
       <scheme val="minor"/>
@@ -207,7 +239,14 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF9C0006"/>
+      <color rgb="FF9C6500"/>
+      <name val="ＭＳ Ｐゴシック"/>
+      <charset val="128"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
       <name val="ＭＳ Ｐゴシック"/>
       <charset val="128"/>
       <scheme val="minor"/>
@@ -215,7 +254,7 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
+      <color rgb="FFFA7D00"/>
       <name val="ＭＳ Ｐゴシック"/>
       <charset val="128"/>
       <scheme val="minor"/>
@@ -224,45 +263,6 @@
       <b/>
       <sz val="15"/>
       <color theme="3"/>
-      <name val="ＭＳ Ｐゴシック"/>
-      <charset val="128"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="ＭＳ Ｐゴシック"/>
-      <charset val="128"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="ＭＳ Ｐゴシック"/>
-      <charset val="128"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="ＭＳ Ｐゴシック"/>
-      <charset val="128"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="ＭＳ Ｐゴシック"/>
-      <charset val="128"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
       <name val="ＭＳ Ｐゴシック"/>
       <charset val="128"/>
       <scheme val="minor"/>
@@ -278,14 +278,14 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color rgb="FFFA7D00"/>
+      <color rgb="FFFFFFFF"/>
       <name val="ＭＳ Ｐゴシック"/>
       <charset val="128"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FFFF0000"/>
+      <color rgb="FF9C0006"/>
       <name val="ＭＳ Ｐゴシック"/>
       <charset val="128"/>
       <scheme val="minor"/>
@@ -300,13 +300,43 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
+        <fgColor rgb="FFFFFFCC"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -318,25 +348,61 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="5"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
+        <fgColor theme="8"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -354,37 +420,55 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="9" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -396,91 +480,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -626,15 +626,6 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="thin">
         <color rgb="FFB2B2B2"/>
       </left>
@@ -646,30 +637,6 @@
       </top>
       <bottom style="thin">
         <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
       </bottom>
       <diagonal/>
     </border>
@@ -715,11 +682,44 @@
     <border>
       <left/>
       <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
       <top style="thin">
         <color theme="4"/>
       </top>
       <bottom style="double">
         <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
       </bottom>
       <diagonal/>
     </border>
@@ -731,7 +731,7 @@
     <xf numFmtId="38" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="27" borderId="17" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="14" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="40" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -740,136 +740,136 @@
     <xf numFmtId="6" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="8" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="14" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="13" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="15" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="18" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="30" borderId="19" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="11" borderId="16" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="13" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="17" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="17" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="30" borderId="17" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="11" borderId="14" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="18" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="22" borderId="16" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="28" borderId="20" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="20" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="19" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -24022,22 +24022,7 @@
                 </a:outerShdw>
               </a:effectLst>
             </a:rPr>
-            <a:t>保存</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="ja-JP" altLang="en-US">
-              <a:solidFill>
-                <a:schemeClr val="tx1"/>
-              </a:solidFill>
-              <a:effectLst>
-                <a:outerShdw blurRad="38100" dist="19050" dir="2700000" algn="tl" rotWithShape="0">
-                  <a:schemeClr val="dk1">
-                    <a:alpha val="40000"/>
-                  </a:schemeClr>
-                </a:outerShdw>
-              </a:effectLst>
-            </a:rPr>
-            <a:t>押下］</a:t>
+            <a:t>保存押下］</a:t>
           </a:r>
           <a:endParaRPr lang="en-US" altLang="ja-JP">
             <a:solidFill>

</xml_diff>

<commit_message>
Implement cooking result feature and improve views
</commit_message>
<xml_diff>
--- a/CurryRecipeManager/docs/01_design/105システムフロー.xlsx
+++ b/CurryRecipeManager/docs/01_design/105システムフロー.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="18551" windowHeight="9840" activeTab="1"/>
+    <workbookView windowWidth="22451" windowHeight="9900" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="レシピ一覧" sheetId="2" r:id="rId1"/>
@@ -141,6 +141,43 @@
     </font>
     <font>
       <sz val="11"/>
+      <color indexed="8"/>
+      <name val="ＭＳ Ｐゴシック"/>
+      <charset val="128"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="ＭＳ Ｐゴシック"/>
+      <charset val="128"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="ＭＳ Ｐゴシック"/>
+      <charset val="128"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="ＭＳ Ｐゴシック"/>
+      <charset val="128"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="ＭＳ Ｐゴシック"/>
+      <charset val="128"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="ＭＳ Ｐゴシック"/>
       <charset val="128"/>
@@ -155,22 +192,8 @@
     </font>
     <font>
       <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="ＭＳ Ｐゴシック"/>
-      <charset val="128"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <sz val="11"/>
-      <color indexed="8"/>
-      <name val="ＭＳ Ｐゴシック"/>
-      <charset val="128"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
+      <color rgb="FF3F3F3F"/>
       <name val="ＭＳ Ｐゴシック"/>
       <charset val="128"/>
       <scheme val="minor"/>
@@ -184,16 +207,25 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="ＭＳ Ｐゴシック"/>
+      <charset val="128"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <b/>
-      <sz val="11"/>
+      <sz val="13"/>
       <color theme="3"/>
       <name val="ＭＳ Ｐゴシック"/>
       <charset val="128"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <u/>
       <sz val="11"/>
-      <color rgb="FFFA7D00"/>
+      <color rgb="FF800080"/>
       <name val="ＭＳ Ｐゴシック"/>
       <charset val="128"/>
       <scheme val="minor"/>
@@ -207,7 +239,14 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF9C0006"/>
+      <color rgb="FF9C6500"/>
+      <name val="ＭＳ Ｐゴシック"/>
+      <charset val="128"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
       <name val="ＭＳ Ｐゴシック"/>
       <charset val="128"/>
       <scheme val="minor"/>
@@ -215,7 +254,7 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
+      <color rgb="FFFA7D00"/>
       <name val="ＭＳ Ｐゴシック"/>
       <charset val="128"/>
       <scheme val="minor"/>
@@ -224,45 +263,6 @@
       <b/>
       <sz val="15"/>
       <color theme="3"/>
-      <name val="ＭＳ Ｐゴシック"/>
-      <charset val="128"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="ＭＳ Ｐゴシック"/>
-      <charset val="128"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="ＭＳ Ｐゴシック"/>
-      <charset val="128"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="ＭＳ Ｐゴシック"/>
-      <charset val="128"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="ＭＳ Ｐゴシック"/>
-      <charset val="128"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
       <name val="ＭＳ Ｐゴシック"/>
       <charset val="128"/>
       <scheme val="minor"/>
@@ -278,14 +278,14 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color rgb="FFFA7D00"/>
+      <color rgb="FFFFFFFF"/>
       <name val="ＭＳ Ｐゴシック"/>
       <charset val="128"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FFFF0000"/>
+      <color rgb="FF9C0006"/>
       <name val="ＭＳ Ｐゴシック"/>
       <charset val="128"/>
       <scheme val="minor"/>
@@ -300,13 +300,43 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
+        <fgColor rgb="FFFFFFCC"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -318,25 +348,61 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="5"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
+        <fgColor theme="8"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -354,37 +420,55 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="9" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -396,91 +480,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -626,15 +626,6 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="thin">
         <color rgb="FFB2B2B2"/>
       </left>
@@ -646,30 +637,6 @@
       </top>
       <bottom style="thin">
         <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
       </bottom>
       <diagonal/>
     </border>
@@ -715,11 +682,44 @@
     <border>
       <left/>
       <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
       <top style="thin">
         <color theme="4"/>
       </top>
       <bottom style="double">
         <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
       </bottom>
       <diagonal/>
     </border>
@@ -731,7 +731,7 @@
     <xf numFmtId="38" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="27" borderId="17" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="14" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="40" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -740,136 +740,136 @@
     <xf numFmtId="6" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="8" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="14" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="13" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="15" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="18" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="30" borderId="19" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="11" borderId="16" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="13" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="17" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="17" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="30" borderId="17" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="11" borderId="14" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="18" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="22" borderId="16" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="28" borderId="20" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="20" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="19" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -24022,22 +24022,7 @@
                 </a:outerShdw>
               </a:effectLst>
             </a:rPr>
-            <a:t>保存</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="ja-JP" altLang="en-US">
-              <a:solidFill>
-                <a:schemeClr val="tx1"/>
-              </a:solidFill>
-              <a:effectLst>
-                <a:outerShdw blurRad="38100" dist="19050" dir="2700000" algn="tl" rotWithShape="0">
-                  <a:schemeClr val="dk1">
-                    <a:alpha val="40000"/>
-                  </a:schemeClr>
-                </a:outerShdw>
-              </a:effectLst>
-            </a:rPr>
-            <a:t>押下］</a:t>
+            <a:t>保存押下］</a:t>
           </a:r>
           <a:endParaRPr lang="en-US" altLang="ja-JP">
             <a:solidFill>

</xml_diff>